<commit_message>
Recortes dos prints centrados em cada elemento
Usados na coluna de print da planilha (Google Sheets e Excel).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QEFj674GE8QAeypzKEbimN
</commit_message>
<xml_diff>
--- a/docs/plano-de-tagueamento-banco-nuzzi.xlsx
+++ b/docs/plano-de-tagueamento-banco-nuzzi.xlsx
@@ -189,7 +189,7 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="4667250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -214,7 +214,7 @@
       <row>2</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -239,7 +239,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="3" name="Image 3" descr="Picture"/>
@@ -264,7 +264,7 @@
       <row>4</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="4" name="Image 4" descr="Picture"/>
@@ -289,7 +289,7 @@
       <row>5</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="5" name="Image 5" descr="Picture"/>
@@ -314,7 +314,7 @@
       <row>6</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="6" name="Image 6" descr="Picture"/>
@@ -339,7 +339,7 @@
       <row>7</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="7" name="Image 7" descr="Picture"/>
@@ -364,7 +364,7 @@
       <row>8</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1981200"/>
     <pic>
       <nvPicPr>
         <cNvPr id="8" name="Image 8" descr="Picture"/>
@@ -389,7 +389,7 @@
       <row>9</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="9" name="Image 9" descr="Picture"/>
@@ -414,7 +414,7 @@
       <row>10</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="10" name="Image 10" descr="Picture"/>
@@ -439,7 +439,7 @@
       <row>11</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="11" name="Image 11" descr="Picture"/>
@@ -464,7 +464,7 @@
       <row>12</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="12" name="Image 12" descr="Picture"/>
@@ -489,7 +489,7 @@
       <row>13</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="13" name="Image 13" descr="Picture"/>
@@ -514,7 +514,7 @@
       <row>14</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="14" name="Image 14" descr="Picture"/>
@@ -539,7 +539,7 @@
       <row>15</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="15" name="Image 15" descr="Picture"/>
@@ -564,7 +564,7 @@
       <row>16</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="4667250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="16" name="Image 16" descr="Picture"/>
@@ -589,7 +589,7 @@
       <row>17</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="17" name="Image 17" descr="Picture"/>
@@ -614,7 +614,7 @@
       <row>18</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1771650"/>
     <pic>
       <nvPicPr>
         <cNvPr id="18" name="Image 18" descr="Picture"/>
@@ -639,7 +639,7 @@
       <row>19</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="19" name="Image 19" descr="Picture"/>
@@ -664,7 +664,7 @@
       <row>20</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="20" name="Image 20" descr="Picture"/>
@@ -689,7 +689,7 @@
       <row>21</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="21" name="Image 21" descr="Picture"/>
@@ -714,7 +714,7 @@
       <row>22</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="22" name="Image 22" descr="Picture"/>
@@ -739,7 +739,7 @@
       <row>23</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="4667250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="23" name="Image 23" descr="Picture"/>
@@ -764,7 +764,7 @@
       <row>24</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="24" name="Image 24" descr="Picture"/>
@@ -789,7 +789,7 @@
       <row>25</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="25" name="Image 25" descr="Picture"/>
@@ -814,7 +814,7 @@
       <row>26</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="26" name="Image 26" descr="Picture"/>
@@ -839,7 +839,7 @@
       <row>27</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="27" name="Image 27" descr="Picture"/>
@@ -864,7 +864,7 @@
       <row>28</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="28" name="Image 28" descr="Picture"/>
@@ -889,7 +889,7 @@
       <row>29</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="29" name="Image 29" descr="Picture"/>
@@ -914,7 +914,7 @@
       <row>30</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="30" name="Image 30" descr="Picture"/>
@@ -939,7 +939,7 @@
       <row>31</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="31" name="Image 31" descr="Picture"/>
@@ -964,7 +964,7 @@
       <row>32</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="32" name="Image 32" descr="Picture"/>
@@ -989,7 +989,7 @@
       <row>33</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="33" name="Image 33" descr="Picture"/>
@@ -1014,7 +1014,7 @@
       <row>34</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="34" name="Image 34" descr="Picture"/>
@@ -1039,7 +1039,7 @@
       <row>35</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="35" name="Image 35" descr="Picture"/>
@@ -1064,7 +1064,7 @@
       <row>36</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="36" name="Image 36" descr="Picture"/>
@@ -1089,7 +1089,7 @@
       <row>37</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="37" name="Image 37" descr="Picture"/>
@@ -1114,7 +1114,7 @@
       <row>38</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="38" name="Image 38" descr="Picture"/>
@@ -1139,7 +1139,7 @@
       <row>39</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="39" name="Image 39" descr="Picture"/>
@@ -1164,7 +1164,7 @@
       <row>40</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="40" name="Image 40" descr="Picture"/>
@@ -1189,7 +1189,7 @@
       <row>41</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="41" name="Image 41" descr="Picture"/>
@@ -1214,7 +1214,7 @@
       <row>42</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="42" name="Image 42" descr="Picture"/>
@@ -1239,7 +1239,7 @@
       <row>43</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="43" name="Image 43" descr="Picture"/>
@@ -1264,7 +1264,7 @@
       <row>44</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="4667250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="44" name="Image 44" descr="Picture"/>
@@ -1289,7 +1289,7 @@
       <row>45</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="45" name="Image 45" descr="Picture"/>
@@ -1314,7 +1314,7 @@
       <row>46</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="4667250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="46" name="Image 46" descr="Picture"/>
@@ -1339,7 +1339,7 @@
       <row>47</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="47" name="Image 47" descr="Picture"/>
@@ -1364,7 +1364,7 @@
       <row>48</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="2609850"/>
     <pic>
       <nvPicPr>
         <cNvPr id="48" name="Image 48" descr="Picture"/>
@@ -1389,7 +1389,7 @@
       <row>49</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="49" name="Image 49" descr="Picture"/>
@@ -1414,7 +1414,7 @@
       <row>50</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="50" name="Image 50" descr="Picture"/>
@@ -1439,7 +1439,7 @@
       <row>51</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="51" name="Image 51" descr="Picture"/>
@@ -1464,7 +1464,7 @@
       <row>52</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="52" name="Image 52" descr="Picture"/>
@@ -1489,7 +1489,7 @@
       <row>53</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="53" name="Image 53" descr="Picture"/>
@@ -1514,7 +1514,7 @@
       <row>54</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="54" name="Image 54" descr="Picture"/>
@@ -1539,7 +1539,7 @@
       <row>55</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="4667250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="55" name="Image 55" descr="Picture"/>
@@ -1564,7 +1564,7 @@
       <row>56</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="56" name="Image 56" descr="Picture"/>
@@ -1589,7 +1589,7 @@
       <row>57</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="57" name="Image 57" descr="Picture"/>
@@ -1614,7 +1614,7 @@
       <row>58</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="58" name="Image 58" descr="Picture"/>
@@ -1639,7 +1639,7 @@
       <row>59</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="59" name="Image 59" descr="Picture"/>
@@ -1664,7 +1664,7 @@
       <row>60</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="60" name="Image 60" descr="Picture"/>
@@ -1689,7 +1689,7 @@
       <row>61</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="61" name="Image 61" descr="Picture"/>
@@ -1714,7 +1714,7 @@
       <row>62</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="4667250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="62" name="Image 62" descr="Picture"/>
@@ -1739,7 +1739,7 @@
       <row>63</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="63" name="Image 63" descr="Picture"/>
@@ -1764,7 +1764,7 @@
       <row>64</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="64" name="Image 64" descr="Picture"/>
@@ -1789,7 +1789,7 @@
       <row>65</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="65" name="Image 65" descr="Picture"/>
@@ -1814,7 +1814,7 @@
       <row>66</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="66" name="Image 66" descr="Picture"/>
@@ -1839,7 +1839,7 @@
       <row>67</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="67" name="Image 67" descr="Picture"/>
@@ -1864,7 +1864,7 @@
       <row>68</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="68" name="Image 68" descr="Picture"/>
@@ -1889,7 +1889,7 @@
       <row>69</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="69" name="Image 69" descr="Picture"/>
@@ -1914,7 +1914,7 @@
       <row>70</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="70" name="Image 70" descr="Picture"/>
@@ -1939,7 +1939,7 @@
       <row>71</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1905000" cy="3895725"/>
+    <ext cx="2286000" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="71" name="Image 71" descr="Picture"/>
@@ -8139,7 +8139,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="312.75" customHeight="1">
+    <row r="2" ht="373.5" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>EL-01</t>
@@ -8188,7 +8188,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr"/>
     </row>
-    <row r="3" ht="312.75" customHeight="1">
+    <row r="3" ht="141" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>EL-02</t>
@@ -8237,7 +8237,7 @@
       </c>
       <c r="K3" s="2" t="inlineStr"/>
     </row>
-    <row r="4" ht="312.75" customHeight="1">
+    <row r="4" ht="141" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>EL-03</t>
@@ -8286,7 +8286,7 @@
       </c>
       <c r="K4" s="2" t="inlineStr"/>
     </row>
-    <row r="5" ht="312.75" customHeight="1">
+    <row r="5" ht="141" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>EL-04</t>
@@ -8335,7 +8335,7 @@
       </c>
       <c r="K5" s="2" t="inlineStr"/>
     </row>
-    <row r="6" ht="312.75" customHeight="1">
+    <row r="6" ht="141" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>EL-05</t>
@@ -8388,7 +8388,7 @@
       </c>
       <c r="K6" s="2" t="inlineStr"/>
     </row>
-    <row r="7" ht="312.75" customHeight="1">
+    <row r="7" ht="141" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>EL-06</t>
@@ -8437,7 +8437,7 @@
       </c>
       <c r="K7" s="2" t="inlineStr"/>
     </row>
-    <row r="8" ht="312.75" customHeight="1">
+    <row r="8" ht="141" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>EL-07</t>
@@ -8490,7 +8490,7 @@
       </c>
       <c r="K8" s="2" t="inlineStr"/>
     </row>
-    <row r="9" ht="312.75" customHeight="1">
+    <row r="9" ht="162" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>EL-08</t>
@@ -8543,7 +8543,7 @@
       </c>
       <c r="K9" s="2" t="inlineStr"/>
     </row>
-    <row r="10" ht="312.75" customHeight="1">
+    <row r="10" ht="141" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>EL-09</t>
@@ -8592,7 +8592,7 @@
       </c>
       <c r="K10" s="2" t="inlineStr"/>
     </row>
-    <row r="11" ht="312.75" customHeight="1">
+    <row r="11" ht="141" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
           <t>EL-10</t>
@@ -8641,7 +8641,7 @@
       </c>
       <c r="K11" s="2" t="inlineStr"/>
     </row>
-    <row r="12" ht="312.75" customHeight="1">
+    <row r="12" ht="141" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t>EL-11</t>
@@ -8690,7 +8690,7 @@
       </c>
       <c r="K12" s="2" t="inlineStr"/>
     </row>
-    <row r="13" ht="312.75" customHeight="1">
+    <row r="13" ht="141" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
           <t>EL-12</t>
@@ -8739,7 +8739,7 @@
       </c>
       <c r="K13" s="2" t="inlineStr"/>
     </row>
-    <row r="14" ht="312.75" customHeight="1">
+    <row r="14" ht="141" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t>EL-13</t>
@@ -8788,7 +8788,7 @@
       </c>
       <c r="K14" s="2" t="inlineStr"/>
     </row>
-    <row r="15" ht="312.75" customHeight="1">
+    <row r="15" ht="141" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>EL-14</t>
@@ -8837,7 +8837,7 @@
       </c>
       <c r="K15" s="2" t="inlineStr"/>
     </row>
-    <row r="16" ht="312.75" customHeight="1">
+    <row r="16" ht="141" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
           <t>EL-15</t>
@@ -8886,7 +8886,7 @@
       </c>
       <c r="K16" s="2" t="inlineStr"/>
     </row>
-    <row r="17" ht="312.75" customHeight="1">
+    <row r="17" ht="373.5" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
           <t>EL-16</t>
@@ -8935,7 +8935,7 @@
       </c>
       <c r="K17" s="2" t="inlineStr"/>
     </row>
-    <row r="18" ht="312.75" customHeight="1">
+    <row r="18" ht="141" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
           <t>EL-17</t>
@@ -8984,7 +8984,7 @@
       </c>
       <c r="K18" s="2" t="inlineStr"/>
     </row>
-    <row r="19" ht="312.75" customHeight="1">
+    <row r="19" ht="145.5" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
           <t>EL-18</t>
@@ -9037,7 +9037,7 @@
       </c>
       <c r="K19" s="2" t="inlineStr"/>
     </row>
-    <row r="20" ht="312.75" customHeight="1">
+    <row r="20" ht="141" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
           <t>EL-19</t>
@@ -9086,7 +9086,7 @@
       </c>
       <c r="K20" s="2" t="inlineStr"/>
     </row>
-    <row r="21" ht="312.75" customHeight="1">
+    <row r="21" ht="141" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
           <t>EL-20</t>
@@ -9135,7 +9135,7 @@
       </c>
       <c r="K21" s="2" t="inlineStr"/>
     </row>
-    <row r="22" ht="312.75" customHeight="1">
+    <row r="22" ht="141" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
           <t>EL-21</t>
@@ -9188,7 +9188,7 @@
       </c>
       <c r="K22" s="2" t="inlineStr"/>
     </row>
-    <row r="23" ht="312.75" customHeight="1">
+    <row r="23" ht="141" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
           <t>EL-22</t>
@@ -9237,7 +9237,7 @@
       </c>
       <c r="K23" s="2" t="inlineStr"/>
     </row>
-    <row r="24" ht="312.75" customHeight="1">
+    <row r="24" ht="373.5" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
           <t>EL-23</t>
@@ -9286,7 +9286,7 @@
       </c>
       <c r="K24" s="2" t="inlineStr"/>
     </row>
-    <row r="25" ht="312.75" customHeight="1">
+    <row r="25" ht="141" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
           <t>EL-24</t>
@@ -9339,7 +9339,7 @@
       </c>
       <c r="K25" s="2" t="inlineStr"/>
     </row>
-    <row r="26" ht="312.75" customHeight="1">
+    <row r="26" ht="141" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
           <t>EL-25</t>
@@ -9388,7 +9388,7 @@
       </c>
       <c r="K26" s="2" t="inlineStr"/>
     </row>
-    <row r="27" ht="312.75" customHeight="1">
+    <row r="27" ht="141" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
           <t>EL-26</t>
@@ -9437,7 +9437,7 @@
       </c>
       <c r="K27" s="2" t="inlineStr"/>
     </row>
-    <row r="28" ht="312.75" customHeight="1">
+    <row r="28" ht="141" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
           <t>EL-27</t>
@@ -9486,7 +9486,7 @@
       </c>
       <c r="K28" s="2" t="inlineStr"/>
     </row>
-    <row r="29" ht="312.75" customHeight="1">
+    <row r="29" ht="141" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
           <t>EL-28</t>
@@ -9535,7 +9535,7 @@
       </c>
       <c r="K29" s="2" t="inlineStr"/>
     </row>
-    <row r="30" ht="312.75" customHeight="1">
+    <row r="30" ht="141" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
           <t>EL-29</t>
@@ -9584,7 +9584,7 @@
       </c>
       <c r="K30" s="2" t="inlineStr"/>
     </row>
-    <row r="31" ht="312.75" customHeight="1">
+    <row r="31" ht="141" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
           <t>EL-30</t>
@@ -9633,7 +9633,7 @@
       </c>
       <c r="K31" s="2" t="inlineStr"/>
     </row>
-    <row r="32" ht="312.75" customHeight="1">
+    <row r="32" ht="141" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
           <t>EL-31</t>
@@ -9682,7 +9682,7 @@
       </c>
       <c r="K32" s="2" t="inlineStr"/>
     </row>
-    <row r="33" ht="312.75" customHeight="1">
+    <row r="33" ht="141" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
           <t>EL-32</t>
@@ -9731,7 +9731,7 @@
       </c>
       <c r="K33" s="2" t="inlineStr"/>
     </row>
-    <row r="34" ht="312.75" customHeight="1">
+    <row r="34" ht="141" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
           <t>EL-33</t>
@@ -9780,7 +9780,7 @@
       </c>
       <c r="K34" s="2" t="inlineStr"/>
     </row>
-    <row r="35" ht="312.75" customHeight="1">
+    <row r="35" ht="141" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
           <t>EL-34</t>
@@ -9829,7 +9829,7 @@
       </c>
       <c r="K35" s="2" t="inlineStr"/>
     </row>
-    <row r="36" ht="312.75" customHeight="1">
+    <row r="36" ht="141" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
           <t>EL-35</t>
@@ -9878,7 +9878,7 @@
       </c>
       <c r="K36" s="2" t="inlineStr"/>
     </row>
-    <row r="37" ht="312.75" customHeight="1">
+    <row r="37" ht="141" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
           <t>EL-36</t>
@@ -9931,7 +9931,7 @@
       </c>
       <c r="K37" s="2" t="inlineStr"/>
     </row>
-    <row r="38" ht="312.75" customHeight="1">
+    <row r="38" ht="141" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
           <t>EL-37</t>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="K38" s="2" t="inlineStr"/>
     </row>
-    <row r="39" ht="312.75" customHeight="1">
+    <row r="39" ht="141" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
           <t>EL-38</t>
@@ -10029,7 +10029,7 @@
       </c>
       <c r="K39" s="2" t="inlineStr"/>
     </row>
-    <row r="40" ht="312.75" customHeight="1">
+    <row r="40" ht="141" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
           <t>EL-39</t>
@@ -10078,7 +10078,7 @@
       </c>
       <c r="K40" s="2" t="inlineStr"/>
     </row>
-    <row r="41" ht="312.75" customHeight="1">
+    <row r="41" ht="141" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
         <is>
           <t>EL-40</t>
@@ -10127,7 +10127,7 @@
       </c>
       <c r="K41" s="2" t="inlineStr"/>
     </row>
-    <row r="42" ht="312.75" customHeight="1">
+    <row r="42" ht="141" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
           <t>EL-41</t>
@@ -10180,7 +10180,7 @@
       </c>
       <c r="K42" s="2" t="inlineStr"/>
     </row>
-    <row r="43" ht="312.75" customHeight="1">
+    <row r="43" ht="141" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
         <is>
           <t>EL-42</t>
@@ -10229,7 +10229,7 @@
       </c>
       <c r="K43" s="2" t="inlineStr"/>
     </row>
-    <row r="44" ht="312.75" customHeight="1">
+    <row r="44" ht="141" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
           <t>EL-43</t>
@@ -10282,7 +10282,7 @@
       </c>
       <c r="K44" s="2" t="inlineStr"/>
     </row>
-    <row r="45" ht="312.75" customHeight="1">
+    <row r="45" ht="373.5" customHeight="1">
       <c r="A45" s="2" t="inlineStr">
         <is>
           <t>EL-44</t>
@@ -10331,7 +10331,7 @@
       </c>
       <c r="K45" s="2" t="inlineStr"/>
     </row>
-    <row r="46" ht="312.75" customHeight="1">
+    <row r="46" ht="141" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
           <t>EL-45</t>
@@ -10384,7 +10384,7 @@
       </c>
       <c r="K46" s="2" t="inlineStr"/>
     </row>
-    <row r="47" ht="312.75" customHeight="1">
+    <row r="47" ht="373.5" customHeight="1">
       <c r="A47" s="2" t="inlineStr">
         <is>
           <t>EL-46</t>
@@ -10433,7 +10433,7 @@
       </c>
       <c r="K47" s="2" t="inlineStr"/>
     </row>
-    <row r="48" ht="312.75" customHeight="1">
+    <row r="48" ht="141" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
         <is>
           <t>EL-47</t>
@@ -10482,7 +10482,7 @@
       </c>
       <c r="K48" s="2" t="inlineStr"/>
     </row>
-    <row r="49" ht="312.75" customHeight="1">
+    <row r="49" ht="211.5" customHeight="1">
       <c r="A49" s="2" t="inlineStr">
         <is>
           <t>EL-48</t>
@@ -10535,7 +10535,7 @@
       </c>
       <c r="K49" s="2" t="inlineStr"/>
     </row>
-    <row r="50" ht="312.75" customHeight="1">
+    <row r="50" ht="141" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
         <is>
           <t>EL-49</t>
@@ -10584,7 +10584,7 @@
       </c>
       <c r="K50" s="2" t="inlineStr"/>
     </row>
-    <row r="51" ht="312.75" customHeight="1">
+    <row r="51" ht="141" customHeight="1">
       <c r="A51" s="2" t="inlineStr">
         <is>
           <t>EL-50</t>
@@ -10637,7 +10637,7 @@
       </c>
       <c r="K51" s="2" t="inlineStr"/>
     </row>
-    <row r="52" ht="312.75" customHeight="1">
+    <row r="52" ht="141" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
         <is>
           <t>EL-51</t>
@@ -10686,7 +10686,7 @@
       </c>
       <c r="K52" s="2" t="inlineStr"/>
     </row>
-    <row r="53" ht="312.75" customHeight="1">
+    <row r="53" ht="141" customHeight="1">
       <c r="A53" s="2" t="inlineStr">
         <is>
           <t>EL-52</t>
@@ -10735,7 +10735,7 @@
       </c>
       <c r="K53" s="2" t="inlineStr"/>
     </row>
-    <row r="54" ht="312.75" customHeight="1">
+    <row r="54" ht="141" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
         <is>
           <t>EL-53</t>
@@ -10784,7 +10784,7 @@
       </c>
       <c r="K54" s="2" t="inlineStr"/>
     </row>
-    <row r="55" ht="312.75" customHeight="1">
+    <row r="55" ht="141" customHeight="1">
       <c r="A55" s="2" t="inlineStr">
         <is>
           <t>EL-54</t>
@@ -10833,7 +10833,7 @@
       </c>
       <c r="K55" s="2" t="inlineStr"/>
     </row>
-    <row r="56" ht="312.75" customHeight="1">
+    <row r="56" ht="373.5" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
         <is>
           <t>EL-55</t>
@@ -10882,7 +10882,7 @@
       </c>
       <c r="K56" s="2" t="inlineStr"/>
     </row>
-    <row r="57" ht="312.75" customHeight="1">
+    <row r="57" ht="141" customHeight="1">
       <c r="A57" s="2" t="inlineStr">
         <is>
           <t>EL-56</t>
@@ -10931,7 +10931,7 @@
       </c>
       <c r="K57" s="2" t="inlineStr"/>
     </row>
-    <row r="58" ht="312.75" customHeight="1">
+    <row r="58" ht="141" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
         <is>
           <t>EL-57</t>
@@ -10980,7 +10980,7 @@
       </c>
       <c r="K58" s="2" t="inlineStr"/>
     </row>
-    <row r="59" ht="312.75" customHeight="1">
+    <row r="59" ht="141" customHeight="1">
       <c r="A59" s="2" t="inlineStr">
         <is>
           <t>EL-58</t>
@@ -11029,7 +11029,7 @@
       </c>
       <c r="K59" s="2" t="inlineStr"/>
     </row>
-    <row r="60" ht="312.75" customHeight="1">
+    <row r="60" ht="141" customHeight="1">
       <c r="A60" s="2" t="inlineStr">
         <is>
           <t>EL-59</t>
@@ -11078,7 +11078,7 @@
       </c>
       <c r="K60" s="2" t="inlineStr"/>
     </row>
-    <row r="61" ht="312.75" customHeight="1">
+    <row r="61" ht="141" customHeight="1">
       <c r="A61" s="2" t="inlineStr">
         <is>
           <t>EL-60</t>
@@ -11127,7 +11127,7 @@
       </c>
       <c r="K61" s="2" t="inlineStr"/>
     </row>
-    <row r="62" ht="312.75" customHeight="1">
+    <row r="62" ht="141" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
         <is>
           <t>EL-61</t>
@@ -11180,7 +11180,7 @@
       </c>
       <c r="K62" s="2" t="inlineStr"/>
     </row>
-    <row r="63" ht="312.75" customHeight="1">
+    <row r="63" ht="373.5" customHeight="1">
       <c r="A63" s="2" t="inlineStr">
         <is>
           <t>EL-62</t>
@@ -11229,7 +11229,7 @@
       </c>
       <c r="K63" s="2" t="inlineStr"/>
     </row>
-    <row r="64" ht="312.75" customHeight="1">
+    <row r="64" ht="141" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
         <is>
           <t>EL-63</t>
@@ -11278,7 +11278,7 @@
       </c>
       <c r="K64" s="2" t="inlineStr"/>
     </row>
-    <row r="65" ht="312.75" customHeight="1">
+    <row r="65" ht="141" customHeight="1">
       <c r="A65" s="2" t="inlineStr">
         <is>
           <t>EL-64</t>
@@ -11327,7 +11327,7 @@
       </c>
       <c r="K65" s="2" t="inlineStr"/>
     </row>
-    <row r="66" ht="312.75" customHeight="1">
+    <row r="66" ht="141" customHeight="1">
       <c r="A66" s="2" t="inlineStr">
         <is>
           <t>EL-65</t>
@@ -11376,7 +11376,7 @@
       </c>
       <c r="K66" s="2" t="inlineStr"/>
     </row>
-    <row r="67" ht="312.75" customHeight="1">
+    <row r="67" ht="141" customHeight="1">
       <c r="A67" s="2" t="inlineStr">
         <is>
           <t>EL-66</t>
@@ -11425,7 +11425,7 @@
       </c>
       <c r="K67" s="2" t="inlineStr"/>
     </row>
-    <row r="68" ht="312.75" customHeight="1">
+    <row r="68" ht="141" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
         <is>
           <t>EL-67</t>
@@ -11478,7 +11478,7 @@
       </c>
       <c r="K68" s="2" t="inlineStr"/>
     </row>
-    <row r="69" ht="312.75" customHeight="1">
+    <row r="69" ht="141" customHeight="1">
       <c r="A69" s="2" t="inlineStr">
         <is>
           <t>EL-68</t>
@@ -11527,7 +11527,7 @@
       </c>
       <c r="K69" s="2" t="inlineStr"/>
     </row>
-    <row r="70" ht="312.75" customHeight="1">
+    <row r="70" ht="141" customHeight="1">
       <c r="A70" s="2" t="inlineStr">
         <is>
           <t>EL-69</t>
@@ -11576,7 +11576,7 @@
       </c>
       <c r="K70" s="2" t="inlineStr"/>
     </row>
-    <row r="71" ht="312.75" customHeight="1">
+    <row r="71" ht="141" customHeight="1">
       <c r="A71" s="2" t="inlineStr">
         <is>
           <t>EL-70</t>
@@ -11625,7 +11625,7 @@
       </c>
       <c r="K71" s="2" t="inlineStr"/>
     </row>
-    <row r="72" ht="312.75" customHeight="1">
+    <row r="72" ht="141" customHeight="1">
       <c r="A72" s="2" t="inlineStr">
         <is>
           <t>EL-71</t>

</xml_diff>